<commit_message>
fix(dataset): close golden case review gaps
</commit_message>
<xml_diff>
--- a/ai-career-dataset/outputs/quality-report/A02_模拟数据与质量报告_v1.2.0.xlsx
+++ b/ai-career-dataset/outputs/quality-report/A02_模拟数据与质量报告_v1.2.0.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Ra49deec2bf9a4358"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规模" sheetId="2" r:id="Re00417c099fe417e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黄金用户" sheetId="3" r:id="R2ae7b0dfd5a54551"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测覆盖" sheetId="4" r:id="R40e7251716f841aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="质量校验" sheetId="5" r:id="R00d095ee49fe4e1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源台账" sheetId="6" r:id="Rdb50addb1f7d4cd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据字典" sheetId="7" r:id="Rb32d7b5a39bf44f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R3b3abd4739754697"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规模" sheetId="2" r:id="R0f1e8dde64234663"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黄金用户" sheetId="3" r:id="R47f71e7625e44859"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测覆盖" sheetId="4" r:id="Rc1acc4764a8c4975"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="质量校验" sheetId="5" r:id="Rea1b1a0435094f38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源台账" sheetId="6" r:id="Rb2abfc86ebb14b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据字典" sheetId="7" r:id="Rb8f51031f5194f8a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -537,7 +537,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0b5e15c664294f2e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0f094596b5a648f9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1536,7 +1536,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d647e7f41204b42"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b2df25e96344948"/>
 </x:worksheet>
 </file>
 
@@ -12260,7 +12260,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E584" s="15" t="str">
-        <x:v>12 golden users, two paths each, eight 8-dimension snapshots each</x:v>
+        <x:v>12 golden users, two paths each, eight 8-dimension snapshots each, and five unique primary milestones</x:v>
       </x:c>
     </x:row>
     <x:row r="585">
@@ -12311,7 +12311,7 @@
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E587" s="15" t="str">
-        <x:v>12 golden users contain ordered learning→project→recalculation→adjustment chain</x:v>
+        <x:v>ordered-chain failures=0, onboarding failures=0, recovery-snapshot failures=0</x:v>
       </x:c>
     </x:row>
     <x:row r="588">
@@ -23306,7 +23306,7 @@
         <x:v>objective</x:v>
       </x:c>
       <x:c r="I344" s="34" t="str">
-        <x:v>4年内达到AI算法工程师独立项目交付水平</x:v>
+        <x:v>4年内补齐“机器学习基础较好，但缺少完整算法项目”相关短板并达到AI算法工程师独立项目交付水平</x:v>
       </x:c>
     </x:row>
     <x:row r="345">
@@ -23826,7 +23826,7 @@
         <x:v>title</x:v>
       </x:c>
       <x:c r="I362" s="34" t="str">
-        <x:v>基础补齐：Python编程</x:v>
+        <x:v>基础复核：机器学习</x:v>
       </x:c>
     </x:row>
     <x:row r="363">
@@ -23855,7 +23855,7 @@
         <x:v>target skill id</x:v>
       </x:c>
       <x:c r="I363" s="34" t="str">
-        <x:v>SKILL-001</x:v>
+        <x:v>SKILL-019</x:v>
       </x:c>
     </x:row>
     <x:row r="364">
@@ -23872,7 +23872,7 @@
         <x:v>target_score</x:v>
       </x:c>
       <x:c r="E364" s="34" t="str">
-        <x:v>integer</x:v>
+        <x:v>number</x:v>
       </x:c>
       <x:c r="F364" s="34" t="str">
         <x:v>是</x:v>
@@ -23884,7 +23884,7 @@
         <x:v>target score</x:v>
       </x:c>
       <x:c r="I364" s="34" t="str">
-        <x:v>82</x:v>
+        <x:v>73.6</x:v>
       </x:c>
     </x:row>
     <x:row r="365">
@@ -23913,7 +23913,7 @@
         <x:v>deliverable</x:v>
       </x:c>
       <x:c r="I365" s="34" t="str">
-        <x:v>测评与学习记录</x:v>
+        <x:v>基线测评与证据复核</x:v>
       </x:c>
     </x:row>
     <x:row r="366">

</xml_diff>